<commit_message>
Stage 8 review fixes: HO-008
</commit_message>
<xml_diff>
--- a/output/archive/Tarnovell_Group/Finance/Integration/2025/Integration_Benefits_Baseline_2025-12.xlsx
+++ b/output/archive/Tarnovell_Group/Finance/Integration/2025/Integration_Benefits_Baseline_2025-12.xlsx
@@ -10,7 +10,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Basis" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Realised" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opportunities" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -165,7 +164,7 @@
   <commentList>
     <comment ref="E7" authorId="0" shapeId="0">
       <text>
-        <t>Realised here means posted and evidenced. Anything not yet in the ledger goes on the Opportunities sheet.</t>
+        <t>Only posted, evidenced cost reductions belong here. A lease notice or approval for a future saving is not a realised benefit.</t>
       </text>
     </comment>
   </commentList>
@@ -461,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -490,12 +489,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Baseline date</t>
+          <t>Baseline issue</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>31/10/2025</t>
+          <t>12/12/2025</t>
         </is>
       </c>
     </row>
@@ -556,7 +555,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Realised savings are only those evidenced in the ledger after the cost has left the firm. Opportunities stay in the second sheet until the Integration Steering Group approves them.</t>
+          <t>Realised savings require an evidenced reduction in cost for the reporting period, net of integration costs. Opportunities stay on the Opportunities sheet until approved and evidenced as delivered.</t>
         </is>
       </c>
     </row>
@@ -569,6 +568,66 @@
       <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Local scientific operations are not reduced by this case. Savings come from shared administration only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Brand line</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Tarnovell Bioscience Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Cut-off</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>30/11/2025; December postings belong to the next baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Calculation</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Compare like-for-like administrative costs for the same period; record local currency, applicable group translation rate and one-off integration costs in the supporting schedule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Exclusions</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Local scientific headcount, client pricing and historical discounts</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Double counting</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Do not repeat benefits already counted in another integration workstream.</t>
         </is>
       </c>
     </row>
@@ -607,12 +666,12 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Scope</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Basis</t>
+          <t>Evidence</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
@@ -622,12 +681,12 @@
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Currency</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>Assumption</t>
+          <t>Calculation assumption</t>
         </is>
       </c>
     </row>
@@ -639,12 +698,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Shared finance processing</t>
+          <t>Realised administrative savings</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Ledger posting</t>
+          <t>Supporting ledger and finance schedule</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -654,12 +713,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Realised</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Headcount in the old finance team not backfilled</t>
+          <t>Use evidenced cost reductions only; net integration costs and retain the local-currency calculation. No amount is reproduced here.</t>
         </is>
       </c>
     </row>
@@ -671,12 +730,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Insurance renewal</t>
+          <t>Realised administrative savings</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Signed renewal</t>
+          <t>Supporting ledger and finance schedule</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -686,12 +745,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Realised</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Single group policy from the 2025 renewal date</t>
+          <t>Use evidenced cost reductions only; net integration costs and retain the local-currency calculation. No amount is reproduced here.</t>
         </is>
       </c>
     </row>
@@ -703,12 +762,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Software licences</t>
+          <t>Realised administrative savings</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Licence register</t>
+          <t>Supporting ledger and finance schedule</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -718,12 +777,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Realised</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Duplicate licences cancelled; no change to user count</t>
+          <t>Use evidenced cost reductions only; net integration costs and retain the local-currency calculation. No amount is reproduced here.</t>
         </is>
       </c>
     </row>
@@ -735,12 +794,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Office consolidation</t>
+          <t>Realised administrative savings</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Lease notice</t>
+          <t>Supporting ledger and finance schedule</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -750,12 +809,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Realised</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Notice period ends in the 2026 financial year</t>
+          <t>Use evidenced cost reductions only; net integration costs and retain the local-currency calculation. No amount is reproduced here.</t>
         </is>
       </c>
     </row>
@@ -767,12 +826,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Shared finance processing</t>
+          <t>Realised administrative savings</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Ledger posting</t>
+          <t>Supporting ledger and finance schedule</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -782,12 +841,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Realised</t>
+          <t>GBP</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Month-end close now run from the group ledger</t>
+          <t>Use evidenced cost reductions only; net integration costs and retain the local-currency calculation. No amount is reproduced here.</t>
         </is>
       </c>
     </row>
@@ -799,27 +858,27 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Travel booking</t>
+          <t>Realised administrative savings</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Booking platform report</t>
+          <t>Supporting ledger and finance schedule</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Aug-Nov 2025</t>
+          <t>Jan-Nov 2025</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Realised</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Only from the date the group booking account went live</t>
+          <t>Use evidenced cost reductions only; net integration costs and retain the local-currency calculation. No amount is reproduced here.</t>
         </is>
       </c>
     </row>
@@ -907,7 +966,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Depends on the HR and payroll consolidation</t>
+          <t>Check remaining payroll-process scope against the consolidated A-F directory.</t>
         </is>
       </c>
     </row>
@@ -971,7 +1030,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Site contract runs to 2027</t>
+          <t>Confirm the site contract term before developing the case.</t>
         </is>
       </c>
     </row>
@@ -1089,7 +1148,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Cost treatment</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1099,112 +1158,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Recorded as a cost of the integration, not a saving</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:C5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Assumption</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>Basis for the figure</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>Reviewed by</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Currency</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Local currency converted at the group rate for the period; no rate is fixed in this baseline</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Andrea Beckett</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Period</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Figures are cut off at 30/11/2025. December postings are picked up in the next baseline</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Andrea Beckett</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Exclusions</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Local scientific headcount, client pricing and historical discounts</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Andrea Beckett</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Double counting</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Items already in the price harmonisation workstream are not counted here</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Sofia Lindervik</t>
+          <t>Deduct shared-services costs from any associated benefit; no saving is claimed for the fee itself.</t>
         </is>
       </c>
     </row>

</xml_diff>